<commit_message>
feat(m9): implement hybrid v2 alarm analysis
</commit_message>
<xml_diff>
--- a/samples/smoke/synthetic_smoke.xlsx
+++ b/samples/smoke/synthetic_smoke.xlsx
@@ -31,7 +31,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.0.0</t>
+          <t>2.0.0</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-01-15T08:20:00+08:00</t>
+          <t>2026-01-15T08:20:05+08:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-01-15T08:20:20+08:00</t>
+          <t>2026-01-15T08:20:25+08:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-01-15T08:20:40+08:00</t>
+          <t>2026-01-15T08:20:45+08:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-01-15T08:21:00+08:00</t>
+          <t>2026-01-15T08:21:05+08:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-01-15T08:21:20+08:00</t>
+          <t>2026-01-15T08:21:25+08:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-01-15T08:21:40+08:00</t>
+          <t>2026-01-15T08:21:45+08:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-01-15T08:22:00+08:00</t>
+          <t>2026-01-15T08:22:05+08:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6294,7 +6294,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-01-15T08:22:20+08:00</t>
+          <t>2026-01-15T08:22:25+08:00</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-01-15T08:22:40+08:00</t>
+          <t>2026-01-15T08:22:45+08:00</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -6622,7 +6622,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-01-15T08:23:00+08:00</t>
+          <t>2026-01-15T08:23:05+08:00</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-01-15T08:23:20+08:00</t>
+          <t>2026-01-15T08:23:25+08:00</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -6950,7 +6950,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-01-15T08:23:40+08:00</t>
+          <t>2026-01-15T08:23:45+08:00</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-01-15T08:24:00+08:00</t>
+          <t>2026-01-15T08:24:05+08:00</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -7278,7 +7278,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-01-15T08:24:20+08:00</t>
+          <t>2026-01-15T08:24:25+08:00</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -7442,7 +7442,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-01-15T08:24:40+08:00</t>
+          <t>2026-01-15T08:24:45+08:00</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7539,17 +7539,17 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -7703,17 +7703,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -7795,7 +7795,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -7872,12 +7872,12 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -7954,12 +7954,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -8036,7 +8036,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -8118,12 +8118,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -8195,7 +8195,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -8205,7 +8205,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_01</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -8446,12 +8446,12 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_02</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -8523,17 +8523,17 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t/>
+          <t>SYNTHETIC_UNIT_02</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -8605,7 +8605,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -8615,7 +8615,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_02</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_02</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -8769,17 +8769,17 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_02</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -8851,17 +8851,17 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_02</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -8933,12 +8933,12 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -9097,17 +9097,17 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_02</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -9261,17 +9261,17 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -9348,7 +9348,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -9430,12 +9430,12 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -9512,12 +9512,12 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -9589,7 +9589,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -9599,7 +9599,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -9681,7 +9681,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -9763,7 +9763,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -9835,17 +9835,17 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -9922,12 +9922,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t/>
+          <t>SYNTHETIC_UNIT_03</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -10004,12 +10004,12 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -10081,17 +10081,17 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -10168,12 +10168,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -10250,12 +10250,12 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -10327,17 +10327,17 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -10501,7 +10501,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -10578,12 +10578,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -10660,12 +10660,12 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -10737,17 +10737,17 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_02</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_04</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -18184,7 +18184,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-01-15T09:40:20+08:00</t>
+          <t>2026-01-15T10:00:00+08:00</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -18204,12 +18204,12 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -18266,7 +18266,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-01-15T09:40:31+08:00</t>
+          <t>2026-01-15T10:00:11+08:00</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -18286,12 +18286,12 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -18348,7 +18348,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-01-15T09:40:42+08:00</t>
+          <t>2026-01-15T10:00:22+08:00</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -18368,12 +18368,12 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -18430,7 +18430,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-01-15T09:40:53+08:00</t>
+          <t>2026-01-15T10:00:33+08:00</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -18450,12 +18450,12 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -18512,7 +18512,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-01-15T09:41:04+08:00</t>
+          <t>2026-01-15T10:00:44+08:00</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -18532,12 +18532,12 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -18594,7 +18594,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-01-15T09:41:15+08:00</t>
+          <t>2026-01-15T10:02:00+08:00</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -18609,17 +18609,17 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -18676,7 +18676,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-01-15T09:41:26+08:00</t>
+          <t>2026-01-15T10:02:11+08:00</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -18691,17 +18691,17 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-01-15T09:41:37+08:00</t>
+          <t>2026-01-15T10:02:22+08:00</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -18773,17 +18773,17 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -18840,7 +18840,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-01-15T09:41:48+08:00</t>
+          <t>2026-01-15T10:02:33+08:00</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -18855,17 +18855,17 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -18922,7 +18922,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-01-15T09:41:59+08:00</t>
+          <t>2026-01-15T10:02:44+08:00</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -18937,17 +18937,17 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -19004,7 +19004,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-01-15T09:42:10+08:00</t>
+          <t>2026-01-15T10:04:00+08:00</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -19029,7 +19029,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -19086,7 +19086,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-01-15T09:42:21+08:00</t>
+          <t>2026-01-15T10:04:11+08:00</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -19111,7 +19111,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -19168,7 +19168,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-01-15T09:42:32+08:00</t>
+          <t>2026-01-15T10:04:22+08:00</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -19193,7 +19193,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -19250,7 +19250,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-01-15T09:42:43+08:00</t>
+          <t>2026-01-15T10:04:33+08:00</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -19332,7 +19332,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-01-15T09:42:54+08:00</t>
+          <t>2026-01-15T10:04:44+08:00</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -19357,7 +19357,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -19414,7 +19414,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-01-15T09:43:05+08:00</t>
+          <t>2026-01-15T10:06:00+08:00</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -19429,17 +19429,17 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -19496,7 +19496,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-01-15T09:43:16+08:00</t>
+          <t>2026-01-15T10:06:11+08:00</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -19511,17 +19511,17 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-01-15T09:43:27+08:00</t>
+          <t>2026-01-15T10:06:22+08:00</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -19593,17 +19593,17 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -19660,7 +19660,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-01-15T09:43:38+08:00</t>
+          <t>2026-01-15T10:06:33+08:00</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -19675,17 +19675,17 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -19742,7 +19742,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-01-15T09:43:49+08:00</t>
+          <t>2026-01-15T10:06:44+08:00</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -19757,17 +19757,17 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_04</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -19824,7 +19824,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-01-15T09:44:00+08:00</t>
+          <t>2026-01-15T10:08:00+08:00</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -19844,7 +19844,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -19906,7 +19906,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-01-15T09:44:11+08:00</t>
+          <t>2026-01-15T10:08:11+08:00</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -19926,7 +19926,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -19988,7 +19988,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-01-15T09:44:22+08:00</t>
+          <t>2026-01-15T10:08:22+08:00</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -20008,7 +20008,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -20070,7 +20070,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-01-15T09:44:33+08:00</t>
+          <t>2026-01-15T10:08:33+08:00</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -20090,7 +20090,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -20152,7 +20152,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-01-15T09:44:44+08:00</t>
+          <t>2026-01-15T10:08:44+08:00</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -20172,7 +20172,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -20234,7 +20234,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-01-15T09:44:55+08:00</t>
+          <t>2026-01-15T10:10:00+08:00</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -20249,17 +20249,17 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-01-15T09:45:06+08:00</t>
+          <t>2026-01-15T10:10:11+08:00</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -20331,17 +20331,17 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-01-15T09:45:17+08:00</t>
+          <t>2026-01-15T10:10:22+08:00</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -20413,17 +20413,17 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -20480,7 +20480,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-01-15T09:45:28+08:00</t>
+          <t>2026-01-15T10:10:33+08:00</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -20495,17 +20495,17 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -20562,7 +20562,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-01-15T09:45:39+08:00</t>
+          <t>2026-01-15T10:10:44+08:00</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -20577,17 +20577,17 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_02</t>
+          <t>SYNTHETIC_SITE_01</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_03</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_06</t>
+          <t>SYNTHETIC_UNIT_05</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -20644,7 +20644,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-01-15T09:45:50+08:00</t>
+          <t>2026-01-15T12:00:00+08:00</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -20659,17 +20659,17 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
@@ -20726,7 +20726,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-01-15T09:46:01+08:00</t>
+          <t>2026-01-15T12:00:11+08:00</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -20741,17 +20741,17 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -20808,7 +20808,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-01-15T09:46:12+08:00</t>
+          <t>2026-01-15T12:00:22+08:00</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -20823,17 +20823,17 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-01-15T09:46:23+08:00</t>
+          <t>2026-01-15T12:00:33+08:00</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -20905,17 +20905,17 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
@@ -20972,7 +20972,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-01-15T09:46:34+08:00</t>
+          <t>2026-01-15T12:00:44+08:00</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -20987,17 +20987,17 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_01</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -21054,7 +21054,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-01-15T09:46:45+08:00</t>
+          <t>2026-01-15T12:02:00+08:00</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -21074,12 +21074,12 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -21136,7 +21136,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-01-15T09:46:56+08:00</t>
+          <t>2026-01-15T12:02:11+08:00</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -21156,12 +21156,12 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -21218,7 +21218,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-01-15T09:47:07+08:00</t>
+          <t>2026-01-15T12:02:22+08:00</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -21238,12 +21238,12 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
@@ -21300,7 +21300,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-01-15T09:47:18+08:00</t>
+          <t>2026-01-15T12:02:33+08:00</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -21320,12 +21320,12 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -21382,7 +21382,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-01-15T09:47:29+08:00</t>
+          <t>2026-01-15T12:02:44+08:00</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -21402,12 +21402,12 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_02</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -21464,7 +21464,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-01-15T09:47:40+08:00</t>
+          <t>2026-01-15T12:04:00+08:00</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -21479,17 +21479,17 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
@@ -21546,7 +21546,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-01-15T09:47:51+08:00</t>
+          <t>2026-01-15T12:04:11+08:00</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -21561,17 +21561,17 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -21628,7 +21628,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-01-15T09:48:02+08:00</t>
+          <t>2026-01-15T12:04:22+08:00</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -21643,17 +21643,17 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -21710,7 +21710,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-01-15T09:48:13+08:00</t>
+          <t>2026-01-15T12:04:33+08:00</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -21725,17 +21725,17 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -21792,7 +21792,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-01-15T09:48:24+08:00</t>
+          <t>2026-01-15T12:04:44+08:00</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -21807,17 +21807,17 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_03</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_03</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -21874,7 +21874,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-01-15T09:48:35+08:00</t>
+          <t>2026-01-15T12:06:00+08:00</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -21899,7 +21899,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -21956,7 +21956,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-01-15T09:48:46+08:00</t>
+          <t>2026-01-15T12:06:11+08:00</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -21981,7 +21981,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
@@ -22038,7 +22038,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-01-15T09:48:57+08:00</t>
+          <t>2026-01-15T12:06:22+08:00</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -22063,7 +22063,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -22120,7 +22120,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-01-15T09:49:08+08:00</t>
+          <t>2026-01-15T12:06:33+08:00</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -22145,7 +22145,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -22202,7 +22202,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-01-15T09:49:19+08:00</t>
+          <t>2026-01-15T12:06:44+08:00</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -22227,7 +22227,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_04</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -22284,7 +22284,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-01-15T09:49:30+08:00</t>
+          <t>2026-01-15T12:08:00+08:00</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -22299,17 +22299,17 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -22366,7 +22366,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-01-15T09:49:41+08:00</t>
+          <t>2026-01-15T12:08:11+08:00</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -22381,17 +22381,17 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
@@ -22448,7 +22448,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-01-15T09:49:52+08:00</t>
+          <t>2026-01-15T12:08:22+08:00</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -22463,17 +22463,17 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
@@ -22530,7 +22530,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-01-15T09:50:03+08:00</t>
+          <t>2026-01-15T12:08:33+08:00</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -22545,17 +22545,17 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
@@ -22612,7 +22612,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-01-15T09:50:14+08:00</t>
+          <t>2026-01-15T12:08:44+08:00</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -22627,17 +22627,17 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>SYNTHETIC_SITE_01</t>
+          <t>SYNTHETIC_SITE_02</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_01</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>SYNTHETIC_UNIT_05</t>
+          <t>SYNTHETIC_UNIT_06</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -22694,7 +22694,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-01-15T09:50:25+08:00</t>
+          <t>2026-01-15T12:10:00+08:00</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -22714,7 +22714,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -22776,7 +22776,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-01-15T09:50:36+08:00</t>
+          <t>2026-01-15T12:10:11+08:00</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -22796,7 +22796,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -22858,7 +22858,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-01-15T09:50:47+08:00</t>
+          <t>2026-01-15T12:10:22+08:00</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -22878,7 +22878,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -22940,7 +22940,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-01-15T09:50:58+08:00</t>
+          <t>2026-01-15T12:10:33+08:00</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -22960,7 +22960,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -23022,7 +23022,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-01-15T09:51:09+08:00</t>
+          <t>2026-01-15T12:10:44+08:00</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -23042,7 +23042,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>SYNTHETIC_AREA_02</t>
+          <t>SYNTHETIC_AREA_04</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">

</xml_diff>